<commit_message>
Update templates, cross-checks, and frontend components
- Fix XBRL template formulas across all 14 template files
- Improve cross-check label matching with fuzzy lookup in util.py
- Enhance frontend: streaming text, results view, token dashboard
- Update base prompt and fill_workbook tool

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XBRL-template-MFRS/01-SOFP-CuNonCu.xlsx
+++ b/XBRL-template-MFRS/01-SOFP-CuNonCu.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -68,8 +68,26 @@
       <family val="0"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -92,6 +110,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
         <bgColor rgb="FFD6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6E4F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,7 +152,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -199,6 +222,21 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -461,12 +499,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="13">
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="28" t="inlineStr">
         <is>
           <t>01/01/YYYY - 31/12/YYYY</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="28" t="inlineStr">
         <is>
           <t>01/01/YYYY - 31/12/YYYY</t>
         </is>
@@ -485,8 +523,8 @@
           <t>Statement of financial position</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n"/>
-      <c r="C4" s="17" t="n"/>
+      <c r="B4" s="25" t="n"/>
+      <c r="C4" s="25" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="13">
       <c r="A5" s="16" t="inlineStr">
@@ -494,8 +532,8 @@
           <t>Statement of financial position</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
+      <c r="B5" s="25" t="n"/>
+      <c r="C5" s="25" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="13">
       <c r="A6" s="16" t="inlineStr">
@@ -503,8 +541,8 @@
           <t>Assets</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n"/>
-      <c r="C6" s="17" t="n"/>
+      <c r="B6" s="25" t="n"/>
+      <c r="C6" s="25" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="13">
       <c r="A7" s="16" t="inlineStr">
@@ -512,8 +550,8 @@
           <t>Non-current assets</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="17" t="n"/>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="25" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="13">
       <c r="A8" s="18" t="inlineStr">
@@ -521,11 +559,11 @@
           <t>*Property, plant and equipment</t>
         </is>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="26">
         <f>'SOFP-Sub-CuNonCu'!B39</f>
         <v/>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="26">
         <f>'SOFP-Sub-CuNonCu'!C39</f>
         <v/>
       </c>
@@ -536,11 +574,11 @@
           <t>*Investment property</t>
         </is>
       </c>
-      <c r="B9" s="19">
+      <c r="B9" s="26">
         <f>'SOFP-Sub-CuNonCu'!B49</f>
         <v/>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="26">
         <f>'SOFP-Sub-CuNonCu'!C49</f>
         <v/>
       </c>
@@ -578,11 +616,11 @@
           <t>*Intangible assets</t>
         </is>
       </c>
-      <c r="B13" s="19">
+      <c r="B13" s="26">
         <f>'SOFP-Sub-CuNonCu'!B69</f>
         <v/>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="26">
         <f>'SOFP-Sub-CuNonCu'!C69</f>
         <v/>
       </c>
@@ -593,11 +631,11 @@
           <t>*Investments in subsidiaries</t>
         </is>
       </c>
-      <c r="B14" s="19">
+      <c r="B14" s="26">
         <f>'SOFP-Sub-CuNonCu'!B77</f>
         <v/>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="26">
         <f>'SOFP-Sub-CuNonCu'!C77</f>
         <v/>
       </c>
@@ -608,11 +646,11 @@
           <t>*Investments in associates</t>
         </is>
       </c>
-      <c r="B15" s="19">
+      <c r="B15" s="26">
         <f>'SOFP-Sub-CuNonCu'!B86</f>
         <v/>
       </c>
-      <c r="C15" s="19">
+      <c r="C15" s="26">
         <f>'SOFP-Sub-CuNonCu'!C86</f>
         <v/>
       </c>
@@ -623,11 +661,11 @@
           <t>*Investments in joint ventures</t>
         </is>
       </c>
-      <c r="B16" s="19">
+      <c r="B16" s="26">
         <f>'SOFP-Sub-CuNonCu'!B95</f>
         <v/>
       </c>
-      <c r="C16" s="19">
+      <c r="C16" s="26">
         <f>'SOFP-Sub-CuNonCu'!C95</f>
         <v/>
       </c>
@@ -647,11 +685,11 @@
           <t>*Trade and other non-current receivables</t>
         </is>
       </c>
-      <c r="B18" s="19">
+      <c r="B18" s="26">
         <f>'SOFP-Sub-CuNonCu'!B120</f>
         <v/>
       </c>
-      <c r="C18" s="19">
+      <c r="C18" s="26">
         <f>'SOFP-Sub-CuNonCu'!C120</f>
         <v/>
       </c>
@@ -680,11 +718,11 @@
           <t>*Derivative financial assets</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="26">
         <f>'SOFP-Sub-CuNonCu'!B129</f>
         <v/>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="26">
         <f>'SOFP-Sub-CuNonCu'!C129</f>
         <v/>
       </c>
@@ -695,11 +733,11 @@
           <t>*Other non-current assets</t>
         </is>
       </c>
-      <c r="B22" s="19">
+      <c r="B22" s="26">
         <f>'SOFP-Sub-CuNonCu'!B198</f>
         <v/>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="26">
         <f>'SOFP-Sub-CuNonCu'!C198</f>
         <v/>
       </c>
@@ -725,8 +763,8 @@
           <t>Current assets</t>
         </is>
       </c>
-      <c r="B24" s="17" t="n"/>
-      <c r="C24" s="17" t="n"/>
+      <c r="B24" s="25" t="n"/>
+      <c r="C24" s="25" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="13">
       <c r="A25" s="18" t="inlineStr">
@@ -734,11 +772,11 @@
           <t>*Inventories</t>
         </is>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="26">
         <f>'SOFP-Sub-CuNonCu'!B136</f>
         <v/>
       </c>
-      <c r="C25" s="19">
+      <c r="C25" s="26">
         <f>'SOFP-Sub-CuNonCu'!C136</f>
         <v/>
       </c>
@@ -776,11 +814,11 @@
           <t>*Trade and other current receivables</t>
         </is>
       </c>
-      <c r="B29" s="19">
+      <c r="B29" s="26">
         <f>'SOFP-Sub-CuNonCu'!B169</f>
         <v/>
       </c>
-      <c r="C29" s="19">
+      <c r="C29" s="26">
         <f>'SOFP-Sub-CuNonCu'!C169</f>
         <v/>
       </c>
@@ -800,11 +838,11 @@
           <t>*Derivative financial assets</t>
         </is>
       </c>
-      <c r="B31" s="19">
+      <c r="B31" s="26">
         <f>'SOFP-Sub-CuNonCu'!B178</f>
         <v/>
       </c>
-      <c r="C31" s="19">
+      <c r="C31" s="26">
         <f>'SOFP-Sub-CuNonCu'!C178</f>
         <v/>
       </c>
@@ -815,11 +853,11 @@
           <t>*Cash and cash equivalents</t>
         </is>
       </c>
-      <c r="B32" s="19">
+      <c r="B32" s="26">
         <f>'SOFP-Sub-CuNonCu'!B193</f>
         <v/>
       </c>
-      <c r="C32" s="19">
+      <c r="C32" s="26">
         <f>'SOFP-Sub-CuNonCu'!C193</f>
         <v/>
       </c>
@@ -893,8 +931,8 @@
           <t>Equity and liabilities</t>
         </is>
       </c>
-      <c r="B38" s="17" t="n"/>
-      <c r="C38" s="17" t="n"/>
+      <c r="B38" s="25" t="n"/>
+      <c r="C38" s="25" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="13">
       <c r="A39" s="16" t="inlineStr">
@@ -902,8 +940,8 @@
           <t>Equity</t>
         </is>
       </c>
-      <c r="B39" s="17" t="n"/>
-      <c r="C39" s="17" t="n"/>
+      <c r="B39" s="25" t="n"/>
+      <c r="C39" s="25" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="13">
       <c r="A40" s="18" t="inlineStr">
@@ -911,11 +949,11 @@
           <t>*Issued capital</t>
         </is>
       </c>
-      <c r="B40" s="19">
+      <c r="B40" s="26">
         <f>'SOFP-Sub-CuNonCu'!B203</f>
         <v/>
       </c>
-      <c r="C40" s="19">
+      <c r="C40" s="26">
         <f>'SOFP-Sub-CuNonCu'!C203</f>
         <v/>
       </c>
@@ -944,11 +982,11 @@
           <t>*Reserves</t>
         </is>
       </c>
-      <c r="B43" s="19">
+      <c r="B43" s="26">
         <f>'SOFP-Sub-CuNonCu'!B222</f>
         <v/>
       </c>
-      <c r="C43" s="19">
+      <c r="C43" s="26">
         <f>'SOFP-Sub-CuNonCu'!C222</f>
         <v/>
       </c>
@@ -974,11 +1012,11 @@
           <t>*Equity - other components</t>
         </is>
       </c>
-      <c r="B45" s="19">
+      <c r="B45" s="26">
         <f>'SOFP-Sub-CuNonCu'!B229</f>
         <v/>
       </c>
-      <c r="C45" s="19">
+      <c r="C45" s="26">
         <f>'SOFP-Sub-CuNonCu'!C229</f>
         <v/>
       </c>
@@ -1013,8 +1051,8 @@
           <t>Liabilities</t>
         </is>
       </c>
-      <c r="B48" s="17" t="n"/>
-      <c r="C48" s="17" t="n"/>
+      <c r="B48" s="25" t="n"/>
+      <c r="C48" s="25" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="13">
       <c r="A49" s="16" t="inlineStr">
@@ -1022,8 +1060,8 @@
           <t>Non-current liabilities</t>
         </is>
       </c>
-      <c r="B49" s="17" t="n"/>
-      <c r="C49" s="17" t="n"/>
+      <c r="B49" s="25" t="n"/>
+      <c r="C49" s="25" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="13">
       <c r="A50" s="20" t="inlineStr">
@@ -1040,11 +1078,11 @@
           <t>*Borrowings</t>
         </is>
       </c>
-      <c r="B51" s="19">
+      <c r="B51" s="26">
         <f>'SOFP-Sub-CuNonCu'!B271</f>
         <v/>
       </c>
-      <c r="C51" s="19">
+      <c r="C51" s="26">
         <f>'SOFP-Sub-CuNonCu'!C271</f>
         <v/>
       </c>
@@ -1064,11 +1102,11 @@
           <t>*Employee benefit liabilities</t>
         </is>
       </c>
-      <c r="B53" s="19">
+      <c r="B53" s="26">
         <f>'SOFP-Sub-CuNonCu'!B280</f>
         <v/>
       </c>
-      <c r="C53" s="19">
+      <c r="C53" s="26">
         <f>'SOFP-Sub-CuNonCu'!C280</f>
         <v/>
       </c>
@@ -1079,11 +1117,11 @@
           <t>*Provisions</t>
         </is>
       </c>
-      <c r="B54" s="19">
+      <c r="B54" s="26">
         <f>'SOFP-Sub-CuNonCu'!B289</f>
         <v/>
       </c>
-      <c r="C54" s="19">
+      <c r="C54" s="26">
         <f>'SOFP-Sub-CuNonCu'!C289</f>
         <v/>
       </c>
@@ -1094,11 +1132,11 @@
           <t>*Trade and other non-current payables</t>
         </is>
       </c>
-      <c r="B55" s="19">
+      <c r="B55" s="26">
         <f>'SOFP-Sub-CuNonCu'!B321</f>
         <v/>
       </c>
-      <c r="C55" s="19">
+      <c r="C55" s="26">
         <f>'SOFP-Sub-CuNonCu'!C321</f>
         <v/>
       </c>
@@ -1127,11 +1165,11 @@
           <t>*Derivative financial liabilities</t>
         </is>
       </c>
-      <c r="B58" s="19">
+      <c r="B58" s="26">
         <f>'SOFP-Sub-CuNonCu'!B336</f>
         <v/>
       </c>
-      <c r="C58" s="19">
+      <c r="C58" s="26">
         <f>'SOFP-Sub-CuNonCu'!C336</f>
         <v/>
       </c>
@@ -1166,8 +1204,8 @@
           <t>Current liabilities</t>
         </is>
       </c>
-      <c r="B61" s="17" t="n"/>
-      <c r="C61" s="17" t="n"/>
+      <c r="B61" s="25" t="n"/>
+      <c r="C61" s="25" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" s="13">
       <c r="A62" s="18" t="inlineStr">
@@ -1175,11 +1213,11 @@
           <t>*Borrowings</t>
         </is>
       </c>
-      <c r="B62" s="19">
+      <c r="B62" s="26">
         <f>'SOFP-Sub-CuNonCu'!B383</f>
         <v/>
       </c>
-      <c r="C62" s="19">
+      <c r="C62" s="26">
         <f>'SOFP-Sub-CuNonCu'!C383</f>
         <v/>
       </c>
@@ -1199,11 +1237,11 @@
           <t>*Employee benefit liabilities</t>
         </is>
       </c>
-      <c r="B64" s="19">
+      <c r="B64" s="26">
         <f>'SOFP-Sub-CuNonCu'!B392</f>
         <v/>
       </c>
-      <c r="C64" s="19">
+      <c r="C64" s="26">
         <f>'SOFP-Sub-CuNonCu'!C392</f>
         <v/>
       </c>
@@ -1214,11 +1252,11 @@
           <t>*Provisions</t>
         </is>
       </c>
-      <c r="B65" s="19">
+      <c r="B65" s="26">
         <f>'SOFP-Sub-CuNonCu'!B401</f>
         <v/>
       </c>
-      <c r="C65" s="19">
+      <c r="C65" s="26">
         <f>'SOFP-Sub-CuNonCu'!C401</f>
         <v/>
       </c>
@@ -1238,11 +1276,11 @@
           <t>*Trade and other current payables</t>
         </is>
       </c>
-      <c r="B67" s="19">
+      <c r="B67" s="26">
         <f>'SOFP-Sub-CuNonCu'!B437</f>
         <v/>
       </c>
-      <c r="C67" s="19">
+      <c r="C67" s="26">
         <f>'SOFP-Sub-CuNonCu'!C437</f>
         <v/>
       </c>
@@ -1262,11 +1300,11 @@
           <t>*Derivative financial liabilities</t>
         </is>
       </c>
-      <c r="B69" s="19">
+      <c r="B69" s="26">
         <f>'SOFP-Sub-CuNonCu'!B452</f>
         <v/>
       </c>
-      <c r="C69" s="19">
+      <c r="C69" s="26">
         <f>'SOFP-Sub-CuNonCu'!C452</f>
         <v/>
       </c>
@@ -1370,12 +1408,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="13">
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="28" t="inlineStr">
         <is>
           <t>01/01/YYYY - 31/12/YYYY</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="28" t="inlineStr">
         <is>
           <t>01/01/YYYY - 31/12/YYYY</t>
         </is>
@@ -1394,8 +1432,8 @@
           <t>Statement on sub-classification of assets, liabilities and equity</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n"/>
-      <c r="C4" s="17" t="n"/>
+      <c r="B4" s="25" t="n"/>
+      <c r="C4" s="25" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="13">
       <c r="A5" s="16" t="inlineStr">
@@ -1403,8 +1441,8 @@
           <t>Statement on sub-classification of assets, liabilities and equity</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
+      <c r="B5" s="25" t="n"/>
+      <c r="C5" s="25" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="13">
       <c r="A6" s="16" t="inlineStr">
@@ -1412,8 +1450,8 @@
           <t>Sub-classification of assets, liabilities and equity</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n"/>
-      <c r="C6" s="17" t="n"/>
+      <c r="B6" s="25" t="n"/>
+      <c r="C6" s="25" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="13">
       <c r="A7" s="16" t="inlineStr">
@@ -1421,8 +1459,8 @@
           <t>Property, plant and equipment</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="17" t="n"/>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="25" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="13">
       <c r="A8" s="16" t="inlineStr">
@@ -1430,8 +1468,8 @@
           <t>Land and buildings</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n"/>
-      <c r="C8" s="17" t="n"/>
+      <c r="B8" s="25" t="n"/>
+      <c r="C8" s="25" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="13">
       <c r="A9" s="16" t="inlineStr">
@@ -1439,8 +1477,8 @@
           <t>Land</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n"/>
-      <c r="C9" s="17" t="n"/>
+      <c r="B9" s="25" t="n"/>
+      <c r="C9" s="25" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="13">
       <c r="A10" s="20" t="inlineStr">
@@ -1490,8 +1528,8 @@
           <t>Buildings</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n"/>
-      <c r="C14" s="17" t="n"/>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="25" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="13">
       <c r="A15" s="20" t="inlineStr">
@@ -1565,8 +1603,8 @@
           <t>Vehicles</t>
         </is>
       </c>
-      <c r="B21" s="17" t="n"/>
-      <c r="C21" s="17" t="n"/>
+      <c r="B21" s="25" t="n"/>
+      <c r="C21" s="25" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="13">
       <c r="A22" s="20" t="inlineStr">
@@ -1748,8 +1786,8 @@
           <t>Investment property</t>
         </is>
       </c>
-      <c r="B40" s="17" t="n"/>
-      <c r="C40" s="17" t="n"/>
+      <c r="B40" s="25" t="n"/>
+      <c r="C40" s="25" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="13">
       <c r="A41" s="16" t="inlineStr">
@@ -1757,8 +1795,8 @@
           <t>Investment properties completed, at carrying value</t>
         </is>
       </c>
-      <c r="B41" s="17" t="n"/>
-      <c r="C41" s="17" t="n"/>
+      <c r="B41" s="25" t="n"/>
+      <c r="C41" s="25" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="13">
       <c r="A42" s="20" t="inlineStr">
@@ -1799,8 +1837,8 @@
           <t>Investment properties under construction or development, at cost</t>
         </is>
       </c>
-      <c r="B45" s="17" t="n"/>
-      <c r="C45" s="17" t="n"/>
+      <c r="B45" s="25" t="n"/>
+      <c r="C45" s="25" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="13">
       <c r="A46" s="20" t="inlineStr">
@@ -1856,8 +1894,8 @@
           <t>Biological assets</t>
         </is>
       </c>
-      <c r="B50" s="17" t="n"/>
-      <c r="C50" s="17" t="n"/>
+      <c r="B50" s="25" t="n"/>
+      <c r="C50" s="25" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1" s="13">
       <c r="A51" s="20" t="inlineStr">
@@ -1898,8 +1936,8 @@
           <t>Intangible assets and goodwill</t>
         </is>
       </c>
-      <c r="B54" s="17" t="n"/>
-      <c r="C54" s="17" t="n"/>
+      <c r="B54" s="25" t="n"/>
+      <c r="C54" s="25" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="13">
       <c r="A55" s="16" t="inlineStr">
@@ -1907,8 +1945,8 @@
           <t>Intangible assets other than goodwill</t>
         </is>
       </c>
-      <c r="B55" s="17" t="n"/>
-      <c r="C55" s="17" t="n"/>
+      <c r="B55" s="25" t="n"/>
+      <c r="C55" s="25" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="13">
       <c r="A56" s="20" t="inlineStr">
@@ -2054,8 +2092,8 @@
           <t>Investments in subsidiaries</t>
         </is>
       </c>
-      <c r="B70" s="17" t="n"/>
-      <c r="C70" s="17" t="n"/>
+      <c r="B70" s="25" t="n"/>
+      <c r="C70" s="25" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1" s="13">
       <c r="A71" s="20" t="inlineStr">
@@ -2132,8 +2170,8 @@
           <t>Investments in associates</t>
         </is>
       </c>
-      <c r="B78" s="17" t="n"/>
-      <c r="C78" s="17" t="n"/>
+      <c r="B78" s="25" t="n"/>
+      <c r="C78" s="25" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1" s="13">
       <c r="A79" s="20" t="inlineStr">
@@ -2219,8 +2257,8 @@
           <t>Investments in joint ventures</t>
         </is>
       </c>
-      <c r="B87" s="17" t="n"/>
-      <c r="C87" s="17" t="n"/>
+      <c r="B87" s="25" t="n"/>
+      <c r="C87" s="25" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1" s="13">
       <c r="A88" s="20" t="inlineStr">
@@ -2306,8 +2344,8 @@
           <t>Trade and other non-current receivables</t>
         </is>
       </c>
-      <c r="B96" s="17" t="n"/>
-      <c r="C96" s="17" t="n"/>
+      <c r="B96" s="25" t="n"/>
+      <c r="C96" s="25" t="n"/>
     </row>
     <row r="97" ht="15" customHeight="1" s="13">
       <c r="A97" s="16" t="inlineStr">
@@ -2315,8 +2353,8 @@
           <t>Non-current trade receivables</t>
         </is>
       </c>
-      <c r="B97" s="17" t="n"/>
-      <c r="C97" s="17" t="n"/>
+      <c r="B97" s="25" t="n"/>
+      <c r="C97" s="25" t="n"/>
     </row>
     <row r="98" ht="15" customHeight="1" s="13">
       <c r="A98" s="20" t="inlineStr">
@@ -2402,8 +2440,8 @@
           <t>Other non-current receivables</t>
         </is>
       </c>
-      <c r="B106" s="17" t="n"/>
-      <c r="C106" s="17" t="n"/>
+      <c r="B106" s="25" t="n"/>
+      <c r="C106" s="25" t="n"/>
     </row>
     <row r="107" ht="15" customHeight="1" s="13">
       <c r="A107" s="16" t="inlineStr">
@@ -2411,8 +2449,8 @@
           <t>Other non-current receivables due from related parties</t>
         </is>
       </c>
-      <c r="B107" s="17" t="n"/>
-      <c r="C107" s="17" t="n"/>
+      <c r="B107" s="25" t="n"/>
+      <c r="C107" s="25" t="n"/>
     </row>
     <row r="108" ht="15" customHeight="1" s="13">
       <c r="A108" s="20" t="inlineStr">
@@ -2480,8 +2518,8 @@
           <t>Non-current non-trade receivables</t>
         </is>
       </c>
-      <c r="B114" s="17" t="n"/>
-      <c r="C114" s="17" t="n"/>
+      <c r="B114" s="25" t="n"/>
+      <c r="C114" s="25" t="n"/>
     </row>
     <row r="115" ht="15" customHeight="1" s="13">
       <c r="A115" s="20" t="inlineStr">
@@ -2561,8 +2599,8 @@
           <t>Non-current derivative financial assets</t>
         </is>
       </c>
-      <c r="B121" s="17" t="n"/>
-      <c r="C121" s="17" t="n"/>
+      <c r="B121" s="25" t="n"/>
+      <c r="C121" s="25" t="n"/>
     </row>
     <row r="122" ht="15" customHeight="1" s="13">
       <c r="A122" s="16" t="inlineStr">
@@ -2570,8 +2608,8 @@
           <t>Non-current derivatives at fair value through profit or loss</t>
         </is>
       </c>
-      <c r="B122" s="17" t="n"/>
-      <c r="C122" s="17" t="n"/>
+      <c r="B122" s="25" t="n"/>
+      <c r="C122" s="25" t="n"/>
     </row>
     <row r="123" ht="15" customHeight="1" s="13">
       <c r="A123" s="20" t="inlineStr">
@@ -2654,8 +2692,8 @@
           <t>Inventories</t>
         </is>
       </c>
-      <c r="B130" s="17" t="n"/>
-      <c r="C130" s="17" t="n"/>
+      <c r="B130" s="25" t="n"/>
+      <c r="C130" s="25" t="n"/>
     </row>
     <row r="131" ht="15" customHeight="1" s="13">
       <c r="A131" s="20" t="inlineStr">
@@ -2723,8 +2761,8 @@
           <t>Trade and other current receivables</t>
         </is>
       </c>
-      <c r="B137" s="17" t="n"/>
-      <c r="C137" s="17" t="n"/>
+      <c r="B137" s="25" t="n"/>
+      <c r="C137" s="25" t="n"/>
     </row>
     <row r="138" ht="15" customHeight="1" s="13">
       <c r="A138" s="16" t="inlineStr">
@@ -2732,8 +2770,8 @@
           <t>Current trade receivables</t>
         </is>
       </c>
-      <c r="B138" s="17" t="n"/>
-      <c r="C138" s="17" t="n"/>
+      <c r="B138" s="25" t="n"/>
+      <c r="C138" s="25" t="n"/>
     </row>
     <row r="139" ht="15" customHeight="1" s="13">
       <c r="A139" s="20" t="inlineStr">
@@ -2837,8 +2875,8 @@
           <t>Other current receivables</t>
         </is>
       </c>
-      <c r="B149" s="17" t="n"/>
-      <c r="C149" s="17" t="n"/>
+      <c r="B149" s="25" t="n"/>
+      <c r="C149" s="25" t="n"/>
     </row>
     <row r="150" ht="15" customHeight="1" s="13">
       <c r="A150" s="16" t="inlineStr">
@@ -2846,8 +2884,8 @@
           <t>Other current receivables due from related parties</t>
         </is>
       </c>
-      <c r="B150" s="17" t="n"/>
-      <c r="C150" s="17" t="n"/>
+      <c r="B150" s="25" t="n"/>
+      <c r="C150" s="25" t="n"/>
     </row>
     <row r="151" ht="15" customHeight="1" s="13">
       <c r="A151" s="20" t="inlineStr">
@@ -2915,8 +2953,8 @@
           <t>Current prepayments and current accrued income</t>
         </is>
       </c>
-      <c r="B157" s="17" t="n"/>
-      <c r="C157" s="17" t="n"/>
+      <c r="B157" s="25" t="n"/>
+      <c r="C157" s="25" t="n"/>
     </row>
     <row r="158" ht="15" customHeight="1" s="13">
       <c r="A158" s="20" t="inlineStr">
@@ -2957,8 +2995,8 @@
           <t>Current non-trade receivables</t>
         </is>
       </c>
-      <c r="B161" s="17" t="n"/>
-      <c r="C161" s="17" t="n"/>
+      <c r="B161" s="25" t="n"/>
+      <c r="C161" s="25" t="n"/>
     </row>
     <row r="162" ht="15" customHeight="1" s="13">
       <c r="A162" s="20" t="inlineStr">
@@ -3056,8 +3094,8 @@
           <t>Current derivative financial assets</t>
         </is>
       </c>
-      <c r="B170" s="17" t="n"/>
-      <c r="C170" s="17" t="n"/>
+      <c r="B170" s="25" t="n"/>
+      <c r="C170" s="25" t="n"/>
     </row>
     <row r="171" ht="15" customHeight="1" s="13">
       <c r="A171" s="16" t="inlineStr">
@@ -3065,8 +3103,8 @@
           <t>Current derivatives at fair value through profit or loss</t>
         </is>
       </c>
-      <c r="B171" s="17" t="n"/>
-      <c r="C171" s="17" t="n"/>
+      <c r="B171" s="25" t="n"/>
+      <c r="C171" s="25" t="n"/>
     </row>
     <row r="172" ht="15" customHeight="1" s="13">
       <c r="A172" s="20" t="inlineStr">
@@ -3149,8 +3187,8 @@
           <t>Cash and cash equivalents</t>
         </is>
       </c>
-      <c r="B179" s="17" t="n"/>
-      <c r="C179" s="17" t="n"/>
+      <c r="B179" s="25" t="n"/>
+      <c r="C179" s="25" t="n"/>
     </row>
     <row r="180" ht="15" customHeight="1" s="13">
       <c r="A180" s="16" t="inlineStr">
@@ -3158,8 +3196,8 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="B180" s="17" t="n"/>
-      <c r="C180" s="17" t="n"/>
+      <c r="B180" s="25" t="n"/>
+      <c r="C180" s="25" t="n"/>
     </row>
     <row r="181" ht="15" customHeight="1" s="13">
       <c r="A181" s="20" t="inlineStr">
@@ -3200,8 +3238,8 @@
           <t>Cash equivalents</t>
         </is>
       </c>
-      <c r="B184" s="17" t="n"/>
-      <c r="C184" s="17" t="n"/>
+      <c r="B184" s="25" t="n"/>
+      <c r="C184" s="25" t="n"/>
     </row>
     <row r="185" ht="15" customHeight="1" s="13">
       <c r="A185" s="20" t="inlineStr">
@@ -3302,8 +3340,8 @@
           <t>Other non-current assets</t>
         </is>
       </c>
-      <c r="B194" s="17" t="n"/>
-      <c r="C194" s="17" t="n"/>
+      <c r="B194" s="25" t="n"/>
+      <c r="C194" s="25" t="n"/>
     </row>
     <row r="195" ht="15" customHeight="1" s="13">
       <c r="A195" s="20" t="inlineStr">
@@ -3353,8 +3391,8 @@
           <t>Issued capital</t>
         </is>
       </c>
-      <c r="B199" s="17" t="n"/>
-      <c r="C199" s="17" t="n"/>
+      <c r="B199" s="25" t="n"/>
+      <c r="C199" s="25" t="n"/>
     </row>
     <row r="200" ht="15" customHeight="1" s="13">
       <c r="A200" s="20" t="inlineStr">
@@ -3404,8 +3442,8 @@
           <t>Reserves</t>
         </is>
       </c>
-      <c r="B204" s="17" t="n"/>
-      <c r="C204" s="17" t="n"/>
+      <c r="B204" s="25" t="n"/>
+      <c r="C204" s="25" t="n"/>
     </row>
     <row r="205" ht="15" customHeight="1" s="13">
       <c r="A205" s="16" t="inlineStr">
@@ -3413,8 +3451,8 @@
           <t>Non-distributable</t>
         </is>
       </c>
-      <c r="B205" s="17" t="n"/>
-      <c r="C205" s="17" t="n"/>
+      <c r="B205" s="25" t="n"/>
+      <c r="C205" s="25" t="n"/>
     </row>
     <row r="206" ht="15" customHeight="1" s="13">
       <c r="A206" s="20" t="inlineStr">
@@ -3509,8 +3547,8 @@
           <t>Distributable</t>
         </is>
       </c>
-      <c r="B215" s="17" t="n"/>
-      <c r="C215" s="17" t="n"/>
+      <c r="B215" s="25" t="n"/>
+      <c r="C215" s="25" t="n"/>
     </row>
     <row r="216" ht="15" customHeight="1" s="13">
       <c r="A216" s="20" t="inlineStr">
@@ -3593,8 +3631,8 @@
           <t>Equity - others components</t>
         </is>
       </c>
-      <c r="B223" s="17" t="n"/>
-      <c r="C223" s="17" t="n"/>
+      <c r="B223" s="25" t="n"/>
+      <c r="C223" s="25" t="n"/>
     </row>
     <row r="224" ht="15" customHeight="1" s="13">
       <c r="A224" s="20" t="inlineStr">
@@ -3662,8 +3700,8 @@
           <t>Non-current borrowings</t>
         </is>
       </c>
-      <c r="B230" s="17" t="n"/>
-      <c r="C230" s="17" t="n"/>
+      <c r="B230" s="25" t="n"/>
+      <c r="C230" s="25" t="n"/>
     </row>
     <row r="231" ht="23.25" customHeight="1" s="13">
       <c r="A231" s="16" t="inlineStr">
@@ -3671,8 +3709,8 @@
           <t>Non-current portion of non-current secured bank loans received</t>
         </is>
       </c>
-      <c r="B231" s="17" t="n"/>
-      <c r="C231" s="17" t="n"/>
+      <c r="B231" s="25" t="n"/>
+      <c r="C231" s="25" t="n"/>
     </row>
     <row r="232" ht="15" customHeight="1" s="13">
       <c r="A232" s="20" t="inlineStr">
@@ -3758,8 +3796,8 @@
           <t>Non-current portion of non-current unsecured bank loans received</t>
         </is>
       </c>
-      <c r="B240" s="17" t="n"/>
-      <c r="C240" s="17" t="n"/>
+      <c r="B240" s="25" t="n"/>
+      <c r="C240" s="25" t="n"/>
     </row>
     <row r="241" ht="15" customHeight="1" s="13">
       <c r="A241" s="20" t="inlineStr">
@@ -3854,8 +3892,8 @@
           <t>Non-current portion of secured bonds, sukuk and loan stock</t>
         </is>
       </c>
-      <c r="B250" s="17" t="n"/>
-      <c r="C250" s="17" t="n"/>
+      <c r="B250" s="25" t="n"/>
+      <c r="C250" s="25" t="n"/>
     </row>
     <row r="251" ht="15" customHeight="1" s="13">
       <c r="A251" s="20" t="inlineStr">
@@ -3923,8 +3961,8 @@
           <t>Non-current portion of unsecured bonds, sukuk and loan stock</t>
         </is>
       </c>
-      <c r="B257" s="17" t="n"/>
-      <c r="C257" s="17" t="n"/>
+      <c r="B257" s="25" t="n"/>
+      <c r="C257" s="25" t="n"/>
     </row>
     <row r="258" ht="15" customHeight="1" s="13">
       <c r="A258" s="20" t="inlineStr">
@@ -3992,8 +4030,8 @@
           <t>Other non-current borrowings</t>
         </is>
       </c>
-      <c r="B264" s="17" t="n"/>
-      <c r="C264" s="17" t="n"/>
+      <c r="B264" s="25" t="n"/>
+      <c r="C264" s="25" t="n"/>
     </row>
     <row r="265" ht="15" customHeight="1" s="13">
       <c r="A265" s="20" t="inlineStr">
@@ -4076,8 +4114,8 @@
           <t>Non-current employee benefit liabilities</t>
         </is>
       </c>
-      <c r="B272" s="17" t="n"/>
-      <c r="C272" s="17" t="n"/>
+      <c r="B272" s="25" t="n"/>
+      <c r="C272" s="25" t="n"/>
     </row>
     <row r="273" ht="15" customHeight="1" s="13">
       <c r="A273" s="20" t="inlineStr">
@@ -4163,8 +4201,8 @@
           <t>Non-current provisions</t>
         </is>
       </c>
-      <c r="B281" s="17" t="n"/>
-      <c r="C281" s="17" t="n"/>
+      <c r="B281" s="25" t="n"/>
+      <c r="C281" s="25" t="n"/>
     </row>
     <row r="282" ht="15" customHeight="1" s="13">
       <c r="A282" s="20" t="inlineStr">
@@ -4250,8 +4288,8 @@
           <t>Trade and other non-current payables</t>
         </is>
       </c>
-      <c r="B290" s="17" t="n"/>
-      <c r="C290" s="17" t="n"/>
+      <c r="B290" s="25" t="n"/>
+      <c r="C290" s="25" t="n"/>
     </row>
     <row r="291" ht="15" customHeight="1" s="13">
       <c r="A291" s="16" t="inlineStr">
@@ -4259,8 +4297,8 @@
           <t>Non-current trade payables</t>
         </is>
       </c>
-      <c r="B291" s="17" t="n"/>
-      <c r="C291" s="17" t="n"/>
+      <c r="B291" s="25" t="n"/>
+      <c r="C291" s="25" t="n"/>
     </row>
     <row r="292" ht="15" customHeight="1" s="13">
       <c r="A292" s="20" t="inlineStr">
@@ -4346,8 +4384,8 @@
           <t>Other non-current payables</t>
         </is>
       </c>
-      <c r="B300" s="17" t="n"/>
-      <c r="C300" s="17" t="n"/>
+      <c r="B300" s="25" t="n"/>
+      <c r="C300" s="25" t="n"/>
     </row>
     <row r="301" ht="15" customHeight="1" s="13">
       <c r="A301" s="16" t="inlineStr">
@@ -4355,8 +4393,8 @@
           <t>Other non-current payables due to related parties</t>
         </is>
       </c>
-      <c r="B301" s="17" t="n"/>
-      <c r="C301" s="17" t="n"/>
+      <c r="B301" s="25" t="n"/>
+      <c r="C301" s="25" t="n"/>
     </row>
     <row r="302" ht="15" customHeight="1" s="13">
       <c r="A302" s="20" t="inlineStr">
@@ -4424,8 +4462,8 @@
           <t>Other payables due to non-controlling interests</t>
         </is>
       </c>
-      <c r="B308" s="17" t="n"/>
-      <c r="C308" s="17" t="n"/>
+      <c r="B308" s="25" t="n"/>
+      <c r="C308" s="25" t="n"/>
     </row>
     <row r="309" ht="15" customHeight="1" s="13">
       <c r="A309" s="20" t="inlineStr">
@@ -4475,8 +4513,8 @@
           <t>Non-current non-trade payables</t>
         </is>
       </c>
-      <c r="B313" s="17" t="n"/>
-      <c r="C313" s="17" t="n"/>
+      <c r="B313" s="25" t="n"/>
+      <c r="C313" s="25" t="n"/>
     </row>
     <row r="314" ht="15" customHeight="1" s="13">
       <c r="A314" s="20" t="inlineStr">
@@ -4544,11 +4582,11 @@
           <t>Other non-current payables</t>
         </is>
       </c>
-      <c r="B320" s="19">
+      <c r="B320" s="27">
         <f>1*B307+1*B312+1*B319</f>
         <v/>
       </c>
-      <c r="C320" s="19">
+      <c r="C320" s="27">
         <f>1*C307+1*C312+1*C319</f>
         <v/>
       </c>
@@ -4574,8 +4612,8 @@
           <t>Non-current derivative financial liabilities</t>
         </is>
       </c>
-      <c r="B322" s="17" t="n"/>
-      <c r="C322" s="17" t="n"/>
+      <c r="B322" s="25" t="n"/>
+      <c r="C322" s="25" t="n"/>
     </row>
     <row r="323" ht="15" customHeight="1" s="13">
       <c r="A323" s="16" t="inlineStr">
@@ -4583,8 +4621,8 @@
           <t>Non-current derivatives at fair value through profit or loss</t>
         </is>
       </c>
-      <c r="B323" s="17" t="n"/>
-      <c r="C323" s="17" t="n"/>
+      <c r="B323" s="25" t="n"/>
+      <c r="C323" s="25" t="n"/>
     </row>
     <row r="324" ht="15" customHeight="1" s="13">
       <c r="A324" s="20" t="inlineStr">
@@ -4643,8 +4681,8 @@
           <t>Non-current Derivates used for hedging</t>
         </is>
       </c>
-      <c r="B329" s="17" t="n"/>
-      <c r="C329" s="17" t="n"/>
+      <c r="B329" s="25" t="n"/>
+      <c r="C329" s="25" t="n"/>
     </row>
     <row r="330" ht="15" customHeight="1" s="13">
       <c r="A330" s="20" t="inlineStr">
@@ -4727,8 +4765,8 @@
           <t>Current borrowings</t>
         </is>
       </c>
-      <c r="B337" s="17" t="n"/>
-      <c r="C337" s="17" t="n"/>
+      <c r="B337" s="25" t="n"/>
+      <c r="C337" s="25" t="n"/>
     </row>
     <row r="338" ht="23.25" customHeight="1" s="13">
       <c r="A338" s="16" t="inlineStr">
@@ -4736,8 +4774,8 @@
           <t>Current secured bank loans received and current portion of non-current secured bank loans received</t>
         </is>
       </c>
-      <c r="B338" s="17" t="n"/>
-      <c r="C338" s="17" t="n"/>
+      <c r="B338" s="25" t="n"/>
+      <c r="C338" s="25" t="n"/>
     </row>
     <row r="339" ht="15" customHeight="1" s="13">
       <c r="A339" s="20" t="inlineStr">
@@ -4850,8 +4888,8 @@
           <t>Current unsecured bank loans received and current portion of non-current unsecured bank loans received</t>
         </is>
       </c>
-      <c r="B350" s="17" t="n"/>
-      <c r="C350" s="17" t="n"/>
+      <c r="B350" s="25" t="n"/>
+      <c r="C350" s="25" t="n"/>
     </row>
     <row r="351" ht="15" customHeight="1" s="13">
       <c r="A351" s="20" t="inlineStr">
@@ -4955,8 +4993,8 @@
           <t>Current portion of secured bonds/sukuk/loan stocks</t>
         </is>
       </c>
-      <c r="B361" s="17" t="n"/>
-      <c r="C361" s="17" t="n"/>
+      <c r="B361" s="25" t="n"/>
+      <c r="C361" s="25" t="n"/>
     </row>
     <row r="362" ht="15" customHeight="1" s="13">
       <c r="A362" s="20" t="inlineStr">
@@ -5024,8 +5062,8 @@
           <t>Current portion of unsecured bonds/sukuk/loan stocks</t>
         </is>
       </c>
-      <c r="B368" s="17" t="n"/>
-      <c r="C368" s="17" t="n"/>
+      <c r="B368" s="25" t="n"/>
+      <c r="C368" s="25" t="n"/>
     </row>
     <row r="369" ht="15" customHeight="1" s="13">
       <c r="A369" s="20" t="inlineStr">
@@ -5093,8 +5131,8 @@
           <t>Other current borrowings</t>
         </is>
       </c>
-      <c r="B375" s="17" t="n"/>
-      <c r="C375" s="17" t="n"/>
+      <c r="B375" s="25" t="n"/>
+      <c r="C375" s="25" t="n"/>
     </row>
     <row r="376" ht="15" customHeight="1" s="13">
       <c r="A376" s="20" t="inlineStr">
@@ -5186,8 +5224,8 @@
           <t>Current employee benefit liabilities</t>
         </is>
       </c>
-      <c r="B384" s="17" t="n"/>
-      <c r="C384" s="17" t="n"/>
+      <c r="B384" s="25" t="n"/>
+      <c r="C384" s="25" t="n"/>
     </row>
     <row r="385" ht="15" customHeight="1" s="13">
       <c r="A385" s="20" t="inlineStr">
@@ -5273,8 +5311,8 @@
           <t>Current provisions</t>
         </is>
       </c>
-      <c r="B393" s="17" t="n"/>
-      <c r="C393" s="17" t="n"/>
+      <c r="B393" s="25" t="n"/>
+      <c r="C393" s="25" t="n"/>
     </row>
     <row r="394" ht="15" customHeight="1" s="13">
       <c r="A394" s="20" t="inlineStr">
@@ -5360,8 +5398,8 @@
           <t>Trade and other current payables</t>
         </is>
       </c>
-      <c r="B402" s="17" t="n"/>
-      <c r="C402" s="17" t="n"/>
+      <c r="B402" s="25" t="n"/>
+      <c r="C402" s="25" t="n"/>
     </row>
     <row r="403" ht="15" customHeight="1" s="13">
       <c r="A403" s="16" t="inlineStr">
@@ -5369,8 +5407,8 @@
           <t>Current trade payables</t>
         </is>
       </c>
-      <c r="B403" s="17" t="n"/>
-      <c r="C403" s="17" t="n"/>
+      <c r="B403" s="25" t="n"/>
+      <c r="C403" s="25" t="n"/>
     </row>
     <row r="404" ht="15" customHeight="1" s="13">
       <c r="A404" s="20" t="inlineStr">
@@ -5465,8 +5503,8 @@
           <t>Other current payables</t>
         </is>
       </c>
-      <c r="B413" s="17" t="n"/>
-      <c r="C413" s="17" t="n"/>
+      <c r="B413" s="25" t="n"/>
+      <c r="C413" s="25" t="n"/>
     </row>
     <row r="414" ht="15" customHeight="1" s="13">
       <c r="A414" s="16" t="inlineStr">
@@ -5474,8 +5512,8 @@
           <t xml:space="preserve"> Other current payables due to related parties</t>
         </is>
       </c>
-      <c r="B414" s="17" t="n"/>
-      <c r="C414" s="17" t="n"/>
+      <c r="B414" s="25" t="n"/>
+      <c r="C414" s="25" t="n"/>
     </row>
     <row r="415" ht="15" customHeight="1" s="13">
       <c r="A415" s="20" t="inlineStr">
@@ -5543,8 +5581,8 @@
           <t>Other payables due to non-controlling interests</t>
         </is>
       </c>
-      <c r="B421" s="17" t="n"/>
-      <c r="C421" s="17" t="n"/>
+      <c r="B421" s="25" t="n"/>
+      <c r="C421" s="25" t="n"/>
     </row>
     <row r="422" ht="15" customHeight="1" s="13">
       <c r="A422" s="20" t="inlineStr">
@@ -5594,8 +5632,8 @@
           <t>Current non-trade payables</t>
         </is>
       </c>
-      <c r="B426" s="17" t="n"/>
-      <c r="C426" s="17" t="n"/>
+      <c r="B426" s="25" t="n"/>
+      <c r="C426" s="25" t="n"/>
     </row>
     <row r="427" ht="15" customHeight="1" s="13">
       <c r="A427" s="20" t="inlineStr">
@@ -5720,8 +5758,8 @@
           <t>Current derivative financial liabilities</t>
         </is>
       </c>
-      <c r="B438" s="17" t="n"/>
-      <c r="C438" s="17" t="n"/>
+      <c r="B438" s="25" t="n"/>
+      <c r="C438" s="25" t="n"/>
     </row>
     <row r="439" ht="15" customHeight="1" s="13">
       <c r="A439" s="16" t="inlineStr">
@@ -5729,8 +5767,8 @@
           <t>Current derivatives at fair value through profit or loss</t>
         </is>
       </c>
-      <c r="B439" s="17" t="n"/>
-      <c r="C439" s="17" t="n"/>
+      <c r="B439" s="25" t="n"/>
+      <c r="C439" s="25" t="n"/>
     </row>
     <row r="440" ht="15" customHeight="1" s="13">
       <c r="A440" s="20" t="inlineStr">
@@ -5789,8 +5827,8 @@
           <t>Current derivatives used for hedging</t>
         </is>
       </c>
-      <c r="B445" s="17" t="n"/>
-      <c r="C445" s="17" t="n"/>
+      <c r="B445" s="25" t="n"/>
+      <c r="C445" s="25" t="n"/>
     </row>
     <row r="446" ht="15" customHeight="1" s="13">
       <c r="A446" s="20" t="inlineStr">

</xml_diff>